<commit_message>
DB verification test modifed
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TargetData.xlsx
+++ b/src/test/resources/testdata/TargetData.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="79">
   <si>
     <t>Key</t>
   </si>
@@ -242,6 +242,15 @@
   </si>
   <si>
     <t>0076</t>
+  </si>
+  <si>
+    <t>uchcawgljc</t>
+  </si>
+  <si>
+    <t>ulgjqaxsgk</t>
+  </si>
+  <si>
+    <t>0112</t>
   </si>
 </sst>
 </file>

</xml_diff>